<commit_message>
remove legacy files and consolidate code
</commit_message>
<xml_diff>
--- a/eval/learning-curve/results/learning_curve_gpt-4o_ft200_incorrect.xlsx
+++ b/eval/learning-curve/results/learning_curve_gpt-4o_ft200_incorrect.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E358"/>
+  <dimension ref="A1:E258"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -521,7 +521,11 @@
           <t>IN</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
@@ -1388,7 +1392,11 @@
           <t>NRTI, NNRTI, INSTI</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="E39" t="n">
         <v>0</v>
       </c>
@@ -1409,7 +1417,11 @@
           <t>EFV, DTG, TDF, 3TC</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr"/>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="E40" t="n">
         <v>0</v>
       </c>
@@ -1428,7 +1440,11 @@
       <c r="C41" t="n">
         <v>51</v>
       </c>
-      <c r="D41" t="inlineStr"/>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E41" t="n">
         <v>0</v>
       </c>
@@ -1449,7 +1465,11 @@
           <t>US</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr"/>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E42" t="n">
         <v>0</v>
       </c>
@@ -1470,7 +1490,11 @@
           <t>2021-2022</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E43" t="n">
         <v>0</v>
       </c>
@@ -1491,7 +1515,11 @@
           <t>RT, IN</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E44" t="n">
         <v>0</v>
       </c>
@@ -2031,7 +2059,11 @@
       <c r="C66" t="n">
         <v>14</v>
       </c>
-      <c r="D66" t="inlineStr"/>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="E66" t="n">
         <v>0</v>
       </c>
@@ -2052,7 +2084,11 @@
           <t>France</t>
         </is>
       </c>
-      <c r="D67" t="inlineStr"/>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="E67" t="n">
         <v>0</v>
       </c>
@@ -2073,7 +2109,11 @@
           <t>2019-2020</t>
         </is>
       </c>
-      <c r="D68" t="inlineStr"/>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="E68" t="n">
         <v>0</v>
       </c>
@@ -2094,7 +2134,11 @@
           <t>RT, IN</t>
         </is>
       </c>
-      <c r="D69" t="inlineStr"/>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="E69" t="n">
         <v>0</v>
       </c>
@@ -2165,7 +2209,11 @@
           <t>NRTI, INSTI</t>
         </is>
       </c>
-      <c r="D72" t="inlineStr"/>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="E72" t="n">
         <v>0</v>
       </c>
@@ -2186,7 +2234,11 @@
           <t>BIC, FTC, TAF</t>
         </is>
       </c>
-      <c r="D73" t="inlineStr"/>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="E73" t="n">
         <v>0</v>
       </c>
@@ -3128,7 +3180,11 @@
           <t>Sanger sequencing</t>
         </is>
       </c>
-      <c r="D111" t="inlineStr"/>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E111" t="n">
         <v>0</v>
       </c>
@@ -4518,7 +4574,11 @@
           <t>RT</t>
         </is>
       </c>
-      <c r="D167" t="inlineStr"/>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
       <c r="E167" t="n">
         <v>0</v>
       </c>
@@ -5212,7 +5272,11 @@
           <t>4559 and 3097</t>
         </is>
       </c>
-      <c r="D195" t="inlineStr"/>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
       <c r="E195" t="n">
         <v>0</v>
       </c>
@@ -6785,2484 +6849,6 @@
         </is>
       </c>
       <c r="E258" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="259">
-      <c r="A259" t="inlineStr">
-        <is>
-          <t>40391923</t>
-        </is>
-      </c>
-      <c r="B259" t="inlineStr">
-        <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
-        </is>
-      </c>
-      <c r="C259" t="n">
-        <v>227</v>
-      </c>
-      <c r="D259" t="inlineStr">
-        <is>
-          <t>234</t>
-        </is>
-      </c>
-      <c r="E259" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="260">
-      <c r="A260" t="inlineStr">
-        <is>
-          <t>40400229</t>
-        </is>
-      </c>
-      <c r="B260" t="inlineStr">
-        <is>
-          <t>From which countries were the sequenced samples obtained?</t>
-        </is>
-      </c>
-      <c r="C260" t="inlineStr">
-        <is>
-          <t>UK</t>
-        </is>
-      </c>
-      <c r="D260" t="inlineStr">
-        <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="E260" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="261">
-      <c r="A261" t="inlineStr">
-        <is>
-          <t>40400229</t>
-        </is>
-      </c>
-      <c r="B261" t="inlineStr">
-        <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
-        </is>
-      </c>
-      <c r="C261" t="inlineStr">
-        <is>
-          <t>RT,IN</t>
-        </is>
-      </c>
-      <c r="D261" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E261" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="262">
-      <c r="A262" t="inlineStr">
-        <is>
-          <t>40400229</t>
-        </is>
-      </c>
-      <c r="B262" t="inlineStr">
-        <is>
-          <t>What method was used for sequencing?</t>
-        </is>
-      </c>
-      <c r="C262" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="D262" t="inlineStr">
-        <is>
-          <t>Stanford algorithm</t>
-        </is>
-      </c>
-      <c r="E262" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="263">
-      <c r="A263" t="inlineStr">
-        <is>
-          <t>40400229</t>
-        </is>
-      </c>
-      <c r="B263" t="inlineStr">
-        <is>
-          <t>What type of samples were sequenced?</t>
-        </is>
-      </c>
-      <c r="C263" t="inlineStr">
-        <is>
-          <t>Plasma</t>
-        </is>
-      </c>
-      <c r="D263" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E263" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="264">
-      <c r="A264" t="inlineStr">
-        <is>
-          <t>40400229</t>
-        </is>
-      </c>
-      <c r="B264" t="inlineStr">
-        <is>
-          <t>Were the patients in the study in a clinical trial?</t>
-        </is>
-      </c>
-      <c r="C264" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D264" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E264" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="265">
-      <c r="A265" t="inlineStr">
-        <is>
-          <t>40431710</t>
-        </is>
-      </c>
-      <c r="B265" t="inlineStr">
-        <is>
-          <t>From what years were the sequenced samples obtained?</t>
-        </is>
-      </c>
-      <c r="C265" t="inlineStr">
-        <is>
-          <t>2006-2024</t>
-        </is>
-      </c>
-      <c r="D265" t="inlineStr">
-        <is>
-          <t>From 1996 to 2024.</t>
-        </is>
-      </c>
-      <c r="E265" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="266">
-      <c r="A266" t="inlineStr">
-        <is>
-          <t>40431710</t>
-        </is>
-      </c>
-      <c r="B266" t="inlineStr">
-        <is>
-          <t>Were the patients in the study in a clinical trial?</t>
-        </is>
-      </c>
-      <c r="C266" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D266" t="inlineStr">
-        <is>
-          <t>Yes.</t>
-        </is>
-      </c>
-      <c r="E266" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="267">
-      <c r="A267" t="inlineStr">
-        <is>
-          <t>40431742</t>
-        </is>
-      </c>
-      <c r="B267" t="inlineStr">
-        <is>
-          <t>Does the paper report in vitro drug susceptibility data?</t>
-        </is>
-      </c>
-      <c r="C267" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D267" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E267" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="268">
-      <c r="A268" t="inlineStr">
-        <is>
-          <t>40431742</t>
-        </is>
-      </c>
-      <c r="B268" t="inlineStr">
-        <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
-        </is>
-      </c>
-      <c r="C268" t="n">
-        <v>1677</v>
-      </c>
-      <c r="D268" t="inlineStr">
-        <is>
-          <t>1667</t>
-        </is>
-      </c>
-      <c r="E268" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="269">
-      <c r="A269" t="inlineStr">
-        <is>
-          <t>40490983</t>
-        </is>
-      </c>
-      <c r="B269" t="inlineStr">
-        <is>
-          <t>What type of samples were sequenced?</t>
-        </is>
-      </c>
-      <c r="C269" t="inlineStr">
-        <is>
-          <t>Plasma</t>
-        </is>
-      </c>
-      <c r="D269" t="inlineStr">
-        <is>
-          <t>Plasma RNA.</t>
-        </is>
-      </c>
-      <c r="E269" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="270">
-      <c r="A270" t="inlineStr">
-        <is>
-          <t>40573423</t>
-        </is>
-      </c>
-      <c r="B270" t="inlineStr">
-        <is>
-          <t>Does the paper report in vitro drug susceptibility data?</t>
-        </is>
-      </c>
-      <c r="C270" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D270" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E270" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="271">
-      <c r="A271" t="inlineStr">
-        <is>
-          <t>40596906</t>
-        </is>
-      </c>
-      <c r="B271" t="inlineStr">
-        <is>
-          <t>What method was used for sequencing?</t>
-        </is>
-      </c>
-      <c r="C271" t="inlineStr">
-        <is>
-          <t>Sanger</t>
-        </is>
-      </c>
-      <c r="D271" t="inlineStr">
-        <is>
-          <t>ViroSeq Genotyping System</t>
-        </is>
-      </c>
-      <c r="E271" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="272">
-      <c r="A272" t="inlineStr">
-        <is>
-          <t>40596906</t>
-        </is>
-      </c>
-      <c r="B272" t="inlineStr">
-        <is>
-          <t>What type of samples were sequenced?</t>
-        </is>
-      </c>
-      <c r="C272" t="inlineStr">
-        <is>
-          <t>Plasma</t>
-        </is>
-      </c>
-      <c r="D272" t="inlineStr">
-        <is>
-          <t>Patient samples</t>
-        </is>
-      </c>
-      <c r="E272" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="273">
-      <c r="A273" t="inlineStr">
-        <is>
-          <t>40596906</t>
-        </is>
-      </c>
-      <c r="B273" t="inlineStr">
-        <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
-        </is>
-      </c>
-      <c r="C273" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="D273" t="inlineStr">
-        <is>
-          <t>Zidovudine (ZDV), Lamivudine (3TC), Nevirapine (NVP), Lopinavir/ritonavir, Efavirenz (EFV), Abacavir (ABC), Didanosine (DDI)</t>
-        </is>
-      </c>
-      <c r="E273" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="274">
-      <c r="A274" t="inlineStr">
-        <is>
-          <t>40713598</t>
-        </is>
-      </c>
-      <c r="B274" t="inlineStr">
-        <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
-        </is>
-      </c>
-      <c r="C274" t="inlineStr">
-        <is>
-          <t>RT</t>
-        </is>
-      </c>
-      <c r="D274" t="inlineStr">
-        <is>
-          <t>HIV-1 pol</t>
-        </is>
-      </c>
-      <c r="E274" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="275">
-      <c r="A275" t="inlineStr">
-        <is>
-          <t>40763144</t>
-        </is>
-      </c>
-      <c r="B275" t="inlineStr">
-        <is>
-          <t>Does the paper report HIV sequences from patient samples?</t>
-        </is>
-      </c>
-      <c r="C275" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D275" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E275" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="276">
-      <c r="A276" t="inlineStr">
-        <is>
-          <t>40763144</t>
-        </is>
-      </c>
-      <c r="B276" t="inlineStr">
-        <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
-        </is>
-      </c>
-      <c r="C276" t="inlineStr">
-        <is>
-          <t>PR, RT, IN</t>
-        </is>
-      </c>
-      <c r="D276" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E276" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="277">
-      <c r="A277" t="inlineStr">
-        <is>
-          <t>40763144</t>
-        </is>
-      </c>
-      <c r="B277" t="inlineStr">
-        <is>
-          <t>What method was used for sequencing?</t>
-        </is>
-      </c>
-      <c r="C277" t="inlineStr">
-        <is>
-          <t>Sanger, NGS</t>
-        </is>
-      </c>
-      <c r="D277" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E277" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="278">
-      <c r="A278" t="inlineStr">
-        <is>
-          <t>40763144</t>
-        </is>
-      </c>
-      <c r="B278" t="inlineStr">
-        <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
-        </is>
-      </c>
-      <c r="C278" t="inlineStr">
-        <is>
-          <t>AZT, ABC, 3TC, TDF, ATV, LPV, RTV, DTG</t>
-        </is>
-      </c>
-      <c r="D278" t="inlineStr">
-        <is>
-          <t>TDF, 3TC, DTG, ABC, ZDV, AZT, LPVr, ATVr</t>
-        </is>
-      </c>
-      <c r="E278" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="279">
-      <c r="A279" t="inlineStr">
-        <is>
-          <t>40779404</t>
-        </is>
-      </c>
-      <c r="B279" t="inlineStr">
-        <is>
-          <t>Does the paper report HIV sequences from patient samples?</t>
-        </is>
-      </c>
-      <c r="C279" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D279" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E279" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="280">
-      <c r="A280" t="inlineStr">
-        <is>
-          <t>40779404</t>
-        </is>
-      </c>
-      <c r="B280" t="inlineStr">
-        <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
-        </is>
-      </c>
-      <c r="C280" t="n">
-        <v>20</v>
-      </c>
-      <c r="D280" t="inlineStr">
-        <is>
-          <t>2028</t>
-        </is>
-      </c>
-      <c r="E280" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="281">
-      <c r="A281" t="inlineStr">
-        <is>
-          <t>40779404</t>
-        </is>
-      </c>
-      <c r="B281" t="inlineStr">
-        <is>
-          <t>What type of samples were sequenced?</t>
-        </is>
-      </c>
-      <c r="C281" t="inlineStr">
-        <is>
-          <t>PBMC</t>
-        </is>
-      </c>
-      <c r="D281" t="inlineStr">
-        <is>
-          <t>Whole blood</t>
-        </is>
-      </c>
-      <c r="E281" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="282">
-      <c r="A282" t="inlineStr">
-        <is>
-          <t>40779404</t>
-        </is>
-      </c>
-      <c r="B282" t="inlineStr">
-        <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
-        </is>
-      </c>
-      <c r="C282" t="inlineStr">
-        <is>
-          <t>TFV (no other ARVs specified; Data in supplementary methods)</t>
-        </is>
-      </c>
-      <c r="D282" t="inlineStr">
-        <is>
-          <t>Tenofovir, Emtricitabine, Instis, NRTIs, NNRTIs</t>
-        </is>
-      </c>
-      <c r="E282" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="283">
-      <c r="A283" t="inlineStr">
-        <is>
-          <t>40857111</t>
-        </is>
-      </c>
-      <c r="B283" t="inlineStr">
-        <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
-        </is>
-      </c>
-      <c r="C283" t="inlineStr">
-        <is>
-          <t>7 (Uncertain)</t>
-        </is>
-      </c>
-      <c r="D283" t="inlineStr">
-        <is>
-          <t>208</t>
-        </is>
-      </c>
-      <c r="E283" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="284">
-      <c r="A284" t="inlineStr">
-        <is>
-          <t>40857111</t>
-        </is>
-      </c>
-      <c r="B284" t="inlineStr">
-        <is>
-          <t>From which countries were the sequenced samples obtained?</t>
-        </is>
-      </c>
-      <c r="C284" t="inlineStr">
-        <is>
-          <t>Not provided (multicenter trial)</t>
-        </is>
-      </c>
-      <c r="D284" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="E284" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="285">
-      <c r="A285" t="inlineStr">
-        <is>
-          <t>40857111</t>
-        </is>
-      </c>
-      <c r="B285" t="inlineStr">
-        <is>
-          <t>From what years were the sequenced samples obtained?</t>
-        </is>
-      </c>
-      <c r="C285" t="inlineStr">
-        <is>
-          <t>Not provided</t>
-        </is>
-      </c>
-      <c r="D285" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="E285" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="286">
-      <c r="A286" t="inlineStr">
-        <is>
-          <t>40857111</t>
-        </is>
-      </c>
-      <c r="B286" t="inlineStr">
-        <is>
-          <t>What method was used for sequencing?</t>
-        </is>
-      </c>
-      <c r="C286" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="D286" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="E286" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="287">
-      <c r="A287" t="inlineStr">
-        <is>
-          <t>40857111</t>
-        </is>
-      </c>
-      <c r="B287" t="inlineStr">
-        <is>
-          <t>What type of samples were sequenced?</t>
-        </is>
-      </c>
-      <c r="C287" t="inlineStr">
-        <is>
-          <t>Plasma</t>
-        </is>
-      </c>
-      <c r="D287" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="E287" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="288">
-      <c r="A288" t="inlineStr">
-        <is>
-          <t>40872801</t>
-        </is>
-      </c>
-      <c r="B288" t="inlineStr">
-        <is>
-          <t>From which countries were the sequenced samples obtained?</t>
-        </is>
-      </c>
-      <c r="C288" t="inlineStr">
-        <is>
-          <t>Tanzania</t>
-        </is>
-      </c>
-      <c r="D288" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E288" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="289">
-      <c r="A289" t="inlineStr">
-        <is>
-          <t>40872801</t>
-        </is>
-      </c>
-      <c r="B289" t="inlineStr">
-        <is>
-          <t>From what years were the sequenced samples obtained?</t>
-        </is>
-      </c>
-      <c r="C289" t="inlineStr">
-        <is>
-          <t>2004-2021</t>
-        </is>
-      </c>
-      <c r="D289" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E289" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="290">
-      <c r="A290" t="inlineStr">
-        <is>
-          <t>40872801</t>
-        </is>
-      </c>
-      <c r="B290" t="inlineStr">
-        <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
-        </is>
-      </c>
-      <c r="C290" t="inlineStr">
-        <is>
-          <t>RT, PR</t>
-        </is>
-      </c>
-      <c r="D290" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E290" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="291">
-      <c r="A291" t="inlineStr">
-        <is>
-          <t>40872801</t>
-        </is>
-      </c>
-      <c r="B291" t="inlineStr">
-        <is>
-          <t>What method was used for sequencing?</t>
-        </is>
-      </c>
-      <c r="C291" t="inlineStr">
-        <is>
-          <t>Sanger</t>
-        </is>
-      </c>
-      <c r="D291" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E291" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="292">
-      <c r="A292" t="inlineStr">
-        <is>
-          <t>40872801</t>
-        </is>
-      </c>
-      <c r="B292" t="inlineStr">
-        <is>
-          <t>What type of samples were sequenced?</t>
-        </is>
-      </c>
-      <c r="C292" t="inlineStr">
-        <is>
-          <t>Plasma</t>
-        </is>
-      </c>
-      <c r="D292" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E292" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="293">
-      <c r="A293" t="inlineStr">
-        <is>
-          <t>40872801</t>
-        </is>
-      </c>
-      <c r="B293" t="inlineStr">
-        <is>
-          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
-        </is>
-      </c>
-      <c r="C293" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D293" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E293" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="294">
-      <c r="A294" t="inlineStr">
-        <is>
-          <t>40872801</t>
-        </is>
-      </c>
-      <c r="B294" t="inlineStr">
-        <is>
-          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
-        </is>
-      </c>
-      <c r="C294" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D294" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E294" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="295">
-      <c r="A295" t="inlineStr">
-        <is>
-          <t>40872801</t>
-        </is>
-      </c>
-      <c r="B295" t="inlineStr">
-        <is>
-          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
-        </is>
-      </c>
-      <c r="C295" t="inlineStr">
-        <is>
-          <t>NRTI, NNRTI, PI</t>
-        </is>
-      </c>
-      <c r="D295" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E295" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="296">
-      <c r="A296" t="inlineStr">
-        <is>
-          <t>40938120</t>
-        </is>
-      </c>
-      <c r="B296" t="inlineStr">
-        <is>
-          <t>Does the paper report HIV sequences from patient samples?</t>
-        </is>
-      </c>
-      <c r="C296" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D296" t="inlineStr">
-        <is>
-          <t>A total of 1,048 eligible pol sequences were analyzed.</t>
-        </is>
-      </c>
-      <c r="E296" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="297">
-      <c r="A297" t="inlineStr">
-        <is>
-          <t>40938120</t>
-        </is>
-      </c>
-      <c r="B297" t="inlineStr">
-        <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
-        </is>
-      </c>
-      <c r="C297" t="n">
-        <v>1048</v>
-      </c>
-      <c r="D297" t="inlineStr">
-        <is>
-          <t>1,260 newly diagnosed, ART-naive individuals.</t>
-        </is>
-      </c>
-      <c r="E297" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="298">
-      <c r="A298" t="inlineStr">
-        <is>
-          <t>40938996</t>
-        </is>
-      </c>
-      <c r="B298" t="inlineStr">
-        <is>
-          <t>Were samples cloned prior to sequencing?</t>
-        </is>
-      </c>
-      <c r="C298" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yes  </t>
-        </is>
-      </c>
-      <c r="D298" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E298" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="299">
-      <c r="A299" t="inlineStr">
-        <is>
-          <t>40938996</t>
-        </is>
-      </c>
-      <c r="B299" t="inlineStr">
-        <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
-        </is>
-      </c>
-      <c r="C299" t="inlineStr">
-        <is>
-          <t>RT, IN, NC, Env</t>
-        </is>
-      </c>
-      <c r="D299" t="inlineStr">
-        <is>
-          <t>NC, IN</t>
-        </is>
-      </c>
-      <c r="E299" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="300">
-      <c r="A300" t="inlineStr">
-        <is>
-          <t>40938996</t>
-        </is>
-      </c>
-      <c r="B300" t="inlineStr">
-        <is>
-          <t>What method was used for sequencing?</t>
-        </is>
-      </c>
-      <c r="C300" t="inlineStr">
-        <is>
-          <t>Sanger, NGS</t>
-        </is>
-      </c>
-      <c r="D300" t="inlineStr">
-        <is>
-          <t>Sanger sequencing</t>
-        </is>
-      </c>
-      <c r="E300" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="301">
-      <c r="A301" t="inlineStr">
-        <is>
-          <t>40965168</t>
-        </is>
-      </c>
-      <c r="B301" t="inlineStr">
-        <is>
-          <t>Does the paper report HIV sequences from patient samples?</t>
-        </is>
-      </c>
-      <c r="C301" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D301" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E301" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="302">
-      <c r="A302" t="inlineStr">
-        <is>
-          <t>40965168</t>
-        </is>
-      </c>
-      <c r="B302" t="inlineStr">
-        <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
-        </is>
-      </c>
-      <c r="C302" t="n">
-        <v>0</v>
-      </c>
-      <c r="D302" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="E302" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="303">
-      <c r="A303" t="inlineStr">
-        <is>
-          <t>40965168</t>
-        </is>
-      </c>
-      <c r="B303" t="inlineStr">
-        <is>
-          <t>What method was used for sequencing?</t>
-        </is>
-      </c>
-      <c r="C303" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="D303" t="inlineStr">
-        <is>
-          <t>Sanger sequencing</t>
-        </is>
-      </c>
-      <c r="E303" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="304">
-      <c r="A304" t="inlineStr">
-        <is>
-          <t>40965168</t>
-        </is>
-      </c>
-      <c r="B304" t="inlineStr">
-        <is>
-          <t>What type of samples were sequenced?</t>
-        </is>
-      </c>
-      <c r="C304" t="inlineStr">
-        <is>
-          <t>Not applicable</t>
-        </is>
-      </c>
-      <c r="D304" t="inlineStr">
-        <is>
-          <t>Plasma samples</t>
-        </is>
-      </c>
-      <c r="E304" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="305">
-      <c r="A305" t="inlineStr">
-        <is>
-          <t>40965168</t>
-        </is>
-      </c>
-      <c r="B305" t="inlineStr">
-        <is>
-          <t>Were the patients in the study in a clinical trial?</t>
-        </is>
-      </c>
-      <c r="C305" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D305" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E305" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="306">
-      <c r="A306" t="inlineStr">
-        <is>
-          <t>40974886</t>
-        </is>
-      </c>
-      <c r="B306" t="inlineStr">
-        <is>
-          <t>From which countries were the sequenced samples obtained?</t>
-        </is>
-      </c>
-      <c r="C306" t="inlineStr">
-        <is>
-          <t>Not provided (multicenter trial)</t>
-        </is>
-      </c>
-      <c r="D306" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="E306" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="307">
-      <c r="A307" t="inlineStr">
-        <is>
-          <t>40974886</t>
-        </is>
-      </c>
-      <c r="B307" t="inlineStr">
-        <is>
-          <t>What method was used for sequencing?</t>
-        </is>
-      </c>
-      <c r="C307" t="inlineStr">
-        <is>
-          <t>NGS</t>
-        </is>
-      </c>
-      <c r="D307" t="inlineStr">
-        <is>
-          <t>Population sequencing</t>
-        </is>
-      </c>
-      <c r="E307" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="308">
-      <c r="A308" t="inlineStr">
-        <is>
-          <t>40974886</t>
-        </is>
-      </c>
-      <c r="B308" t="inlineStr">
-        <is>
-          <t>What type of samples were sequenced?</t>
-        </is>
-      </c>
-      <c r="C308" t="inlineStr">
-        <is>
-          <t>PBMC (Whole blood OK)</t>
-        </is>
-      </c>
-      <c r="D308" t="inlineStr">
-        <is>
-          <t>Whole blood</t>
-        </is>
-      </c>
-      <c r="E308" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="309">
-      <c r="A309" t="inlineStr">
-        <is>
-          <t>40974886</t>
-        </is>
-      </c>
-      <c r="B309" t="inlineStr">
-        <is>
-          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
-        </is>
-      </c>
-      <c r="C309" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D309" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E309" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="310">
-      <c r="A310" t="inlineStr">
-        <is>
-          <t>41004608</t>
-        </is>
-      </c>
-      <c r="B310" t="inlineStr">
-        <is>
-          <t>From which countries were the sequenced samples obtained?</t>
-        </is>
-      </c>
-      <c r="C310" t="inlineStr">
-        <is>
-          <t>UK</t>
-        </is>
-      </c>
-      <c r="D310" t="inlineStr">
-        <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="E310" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="311">
-      <c r="A311" t="inlineStr">
-        <is>
-          <t>41004608</t>
-        </is>
-      </c>
-      <c r="B311" t="inlineStr">
-        <is>
-          <t>What method was used for sequencing?</t>
-        </is>
-      </c>
-      <c r="C311" t="inlineStr">
-        <is>
-          <t>NGS</t>
-        </is>
-      </c>
-      <c r="D311" t="inlineStr">
-        <is>
-          <t>Whole genome sequencing</t>
-        </is>
-      </c>
-      <c r="E311" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="312">
-      <c r="A312" t="inlineStr">
-        <is>
-          <t>41004608</t>
-        </is>
-      </c>
-      <c r="B312" t="inlineStr">
-        <is>
-          <t>What type of samples were sequenced?</t>
-        </is>
-      </c>
-      <c r="C312" t="inlineStr">
-        <is>
-          <t>Plasma</t>
-        </is>
-      </c>
-      <c r="D312" t="inlineStr">
-        <is>
-          <t>Clinical specimens</t>
-        </is>
-      </c>
-      <c r="E312" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="313">
-      <c r="A313" t="inlineStr">
-        <is>
-          <t>41012586</t>
-        </is>
-      </c>
-      <c r="B313" t="inlineStr">
-        <is>
-          <t>Does the paper report HIV sequences from patient samples?</t>
-        </is>
-      </c>
-      <c r="C313" t="inlineStr">
-        <is>
-          <t>Yes (Only past sequences)</t>
-        </is>
-      </c>
-      <c r="D313" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E313" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="314">
-      <c r="A314" t="inlineStr">
-        <is>
-          <t>41012586</t>
-        </is>
-      </c>
-      <c r="B314" t="inlineStr">
-        <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
-        </is>
-      </c>
-      <c r="C314" t="inlineStr">
-        <is>
-          <t>249 (uncertain)</t>
-        </is>
-      </c>
-      <c r="D314" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E314" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="315">
-      <c r="A315" t="inlineStr">
-        <is>
-          <t>41012586</t>
-        </is>
-      </c>
-      <c r="B315" t="inlineStr">
-        <is>
-          <t>From which countries were the sequenced samples obtained?</t>
-        </is>
-      </c>
-      <c r="C315" t="inlineStr">
-        <is>
-          <t>Italy</t>
-        </is>
-      </c>
-      <c r="D315" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E315" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="316">
-      <c r="A316" t="inlineStr">
-        <is>
-          <t>41012586</t>
-        </is>
-      </c>
-      <c r="B316" t="inlineStr">
-        <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
-        </is>
-      </c>
-      <c r="C316" t="inlineStr">
-        <is>
-          <t>PR, RT, IN (presumably)</t>
-        </is>
-      </c>
-      <c r="D316" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E316" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="317">
-      <c r="A317" t="inlineStr">
-        <is>
-          <t>41012586</t>
-        </is>
-      </c>
-      <c r="B317" t="inlineStr">
-        <is>
-          <t>What type of samples were sequenced?</t>
-        </is>
-      </c>
-      <c r="C317" t="inlineStr">
-        <is>
-          <t>Plasma (presumably)</t>
-        </is>
-      </c>
-      <c r="D317" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E317" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="318">
-      <c r="A318" t="inlineStr">
-        <is>
-          <t>41012586</t>
-        </is>
-      </c>
-      <c r="B318" t="inlineStr">
-        <is>
-          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
-        </is>
-      </c>
-      <c r="C318" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D318" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E318" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="319">
-      <c r="A319" t="inlineStr">
-        <is>
-          <t>41012586</t>
-        </is>
-      </c>
-      <c r="B319" t="inlineStr">
-        <is>
-          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
-        </is>
-      </c>
-      <c r="C319" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D319" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E319" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="320">
-      <c r="A320" t="inlineStr">
-        <is>
-          <t>41012586</t>
-        </is>
-      </c>
-      <c r="B320" t="inlineStr">
-        <is>
-          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
-        </is>
-      </c>
-      <c r="C320" t="inlineStr">
-        <is>
-          <t>PI, INSTI, NRTI (presumably)</t>
-        </is>
-      </c>
-      <c r="D320" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E320" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="321">
-      <c r="A321" t="inlineStr">
-        <is>
-          <t>41012586</t>
-        </is>
-      </c>
-      <c r="B321" t="inlineStr">
-        <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
-        </is>
-      </c>
-      <c r="C321" t="inlineStr">
-        <is>
-          <t>DTG, DRV/r</t>
-        </is>
-      </c>
-      <c r="D321" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E321" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="322">
-      <c r="A322" t="inlineStr">
-        <is>
-          <t>41023944</t>
-        </is>
-      </c>
-      <c r="B322" t="inlineStr">
-        <is>
-          <t>From what years were the sequenced samples obtained?</t>
-        </is>
-      </c>
-      <c r="C322" t="inlineStr">
-        <is>
-          <t>2022-2024</t>
-        </is>
-      </c>
-      <c r="D322" t="inlineStr">
-        <is>
-          <t>2023-2024</t>
-        </is>
-      </c>
-      <c r="E322" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="323">
-      <c r="A323" t="inlineStr">
-        <is>
-          <t>41023944</t>
-        </is>
-      </c>
-      <c r="B323" t="inlineStr">
-        <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
-        </is>
-      </c>
-      <c r="C323" t="inlineStr">
-        <is>
-          <t>DTG (no other ARVs specified)</t>
-        </is>
-      </c>
-      <c r="D323" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
-      <c r="E323" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="324">
-      <c r="A324" t="inlineStr">
-        <is>
-          <t>41056006</t>
-        </is>
-      </c>
-      <c r="B324" t="inlineStr">
-        <is>
-          <t>Does the paper report HIV sequences from patient samples?</t>
-        </is>
-      </c>
-      <c r="C324" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D324" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E324" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="325">
-      <c r="A325" t="inlineStr">
-        <is>
-          <t>41056006</t>
-        </is>
-      </c>
-      <c r="B325" t="inlineStr">
-        <is>
-          <t>From which countries were the sequenced samples obtained?</t>
-        </is>
-      </c>
-      <c r="C325" t="inlineStr">
-        <is>
-          <t>Not provided (multicenter trial)</t>
-        </is>
-      </c>
-      <c r="D325" t="inlineStr">
-        <is>
-          <t>USA, Dominican Republic</t>
-        </is>
-      </c>
-      <c r="E325" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="326">
-      <c r="A326" t="inlineStr">
-        <is>
-          <t>41056006</t>
-        </is>
-      </c>
-      <c r="B326" t="inlineStr">
-        <is>
-          <t>From what years were the sequenced samples obtained?</t>
-        </is>
-      </c>
-      <c r="C326" t="inlineStr">
-        <is>
-          <t>Not provided</t>
-        </is>
-      </c>
-      <c r="D326" t="inlineStr">
-        <is>
-          <t>2019-2020</t>
-        </is>
-      </c>
-      <c r="E326" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="327">
-      <c r="A327" t="inlineStr">
-        <is>
-          <t>41056006</t>
-        </is>
-      </c>
-      <c r="B327" t="inlineStr">
-        <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
-        </is>
-      </c>
-      <c r="C327" t="inlineStr">
-        <is>
-          <t>CA</t>
-        </is>
-      </c>
-      <c r="D327" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E327" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="328">
-      <c r="A328" t="inlineStr">
-        <is>
-          <t>41056006</t>
-        </is>
-      </c>
-      <c r="B328" t="inlineStr">
-        <is>
-          <t>What method was used for sequencing?</t>
-        </is>
-      </c>
-      <c r="C328" t="inlineStr">
-        <is>
-          <t>Sanger</t>
-        </is>
-      </c>
-      <c r="D328" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E328" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="329">
-      <c r="A329" t="inlineStr">
-        <is>
-          <t>41056006</t>
-        </is>
-      </c>
-      <c r="B329" t="inlineStr">
-        <is>
-          <t>What type of samples were sequenced?</t>
-        </is>
-      </c>
-      <c r="C329" t="inlineStr">
-        <is>
-          <t>Plasma</t>
-        </is>
-      </c>
-      <c r="D329" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E329" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="330">
-      <c r="A330" t="inlineStr">
-        <is>
-          <t>41057785</t>
-        </is>
-      </c>
-      <c r="B330" t="inlineStr">
-        <is>
-          <t>Does the paper report HIV sequences from patient samples?</t>
-        </is>
-      </c>
-      <c r="C330" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D330" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E330" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="331">
-      <c r="A331" t="inlineStr">
-        <is>
-          <t>41057785</t>
-        </is>
-      </c>
-      <c r="B331" t="inlineStr">
-        <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
-        </is>
-      </c>
-      <c r="C331" t="n">
-        <v>235</v>
-      </c>
-      <c r="D331" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E331" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="332">
-      <c r="A332" t="inlineStr">
-        <is>
-          <t>41057785</t>
-        </is>
-      </c>
-      <c r="B332" t="inlineStr">
-        <is>
-          <t>From which countries were the sequenced samples obtained?</t>
-        </is>
-      </c>
-      <c r="C332" t="inlineStr">
-        <is>
-          <t>Uganda</t>
-        </is>
-      </c>
-      <c r="D332" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E332" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="333">
-      <c r="A333" t="inlineStr">
-        <is>
-          <t>41057785</t>
-        </is>
-      </c>
-      <c r="B333" t="inlineStr">
-        <is>
-          <t>From what years were the sequenced samples obtained?</t>
-        </is>
-      </c>
-      <c r="C333" t="inlineStr">
-        <is>
-          <t>2018-2023</t>
-        </is>
-      </c>
-      <c r="D333" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E333" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="334">
-      <c r="A334" t="inlineStr">
-        <is>
-          <t>41057785</t>
-        </is>
-      </c>
-      <c r="B334" t="inlineStr">
-        <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
-        </is>
-      </c>
-      <c r="C334" t="inlineStr">
-        <is>
-          <t>RT,PR,IN</t>
-        </is>
-      </c>
-      <c r="D334" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E334" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="335">
-      <c r="A335" t="inlineStr">
-        <is>
-          <t>41057785</t>
-        </is>
-      </c>
-      <c r="B335" t="inlineStr">
-        <is>
-          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
-        </is>
-      </c>
-      <c r="C335" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D335" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E335" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="336">
-      <c r="A336" t="inlineStr">
-        <is>
-          <t>41057785</t>
-        </is>
-      </c>
-      <c r="B336" t="inlineStr">
-        <is>
-          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
-        </is>
-      </c>
-      <c r="C336" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D336" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E336" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="337">
-      <c r="A337" t="inlineStr">
-        <is>
-          <t>41057785</t>
-        </is>
-      </c>
-      <c r="B337" t="inlineStr">
-        <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
-        </is>
-      </c>
-      <c r="C337" t="inlineStr">
-        <is>
-          <t>ABC, AZT, D4T, TDF, ETR, NVP, EFV, LPV, DRV/r, DTG</t>
-        </is>
-      </c>
-      <c r="D337" t="inlineStr">
-        <is>
-          <t>AZT, D4T, TDF, ABC, DTG</t>
-        </is>
-      </c>
-      <c r="E337" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="338">
-      <c r="A338" t="inlineStr">
-        <is>
-          <t>41088231</t>
-        </is>
-      </c>
-      <c r="B338" t="inlineStr">
-        <is>
-          <t>Were samples cloned prior to sequencing?</t>
-        </is>
-      </c>
-      <c r="C338" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D338" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E338" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="339">
-      <c r="A339" t="inlineStr">
-        <is>
-          <t>41088231</t>
-        </is>
-      </c>
-      <c r="B339" t="inlineStr">
-        <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
-        </is>
-      </c>
-      <c r="C339" t="inlineStr">
-        <is>
-          <t>Whole genome</t>
-        </is>
-      </c>
-      <c r="D339" t="inlineStr">
-        <is>
-          <t>Near full-length genome (NFLG), partial pol gene, vif, env</t>
-        </is>
-      </c>
-      <c r="E339" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="340">
-      <c r="A340" t="inlineStr">
-        <is>
-          <t>41091504</t>
-        </is>
-      </c>
-      <c r="B340" t="inlineStr">
-        <is>
-          <t>Were samples cloned prior to sequencing?</t>
-        </is>
-      </c>
-      <c r="C340" t="inlineStr">
-        <is>
-          <t>Yes (site-directed mutants)</t>
-        </is>
-      </c>
-      <c r="D340" t="inlineStr"/>
-      <c r="E340" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="341">
-      <c r="A341" t="inlineStr">
-        <is>
-          <t>41091504</t>
-        </is>
-      </c>
-      <c r="B341" t="inlineStr">
-        <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
-        </is>
-      </c>
-      <c r="C341" t="inlineStr">
-        <is>
-          <t>PR</t>
-        </is>
-      </c>
-      <c r="D341" t="inlineStr"/>
-      <c r="E341" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="342">
-      <c r="A342" t="inlineStr">
-        <is>
-          <t>41093949</t>
-        </is>
-      </c>
-      <c r="B342" t="inlineStr">
-        <is>
-          <t>From which countries were the sequenced samples obtained?</t>
-        </is>
-      </c>
-      <c r="C342" t="inlineStr">
-        <is>
-          <t>Not applicable.</t>
-        </is>
-      </c>
-      <c r="D342" t="inlineStr">
-        <is>
-          <t>China, United States</t>
-        </is>
-      </c>
-      <c r="E342" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="343">
-      <c r="A343" t="inlineStr">
-        <is>
-          <t>41093949</t>
-        </is>
-      </c>
-      <c r="B343" t="inlineStr">
-        <is>
-          <t>From what years were the sequenced samples obtained?</t>
-        </is>
-      </c>
-      <c r="C343" t="inlineStr">
-        <is>
-          <t>Not applicable.</t>
-        </is>
-      </c>
-      <c r="D343" t="inlineStr">
-        <is>
-          <t>1978 to 2023</t>
-        </is>
-      </c>
-      <c r="E343" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="344">
-      <c r="A344" t="inlineStr">
-        <is>
-          <t>41093949</t>
-        </is>
-      </c>
-      <c r="B344" t="inlineStr">
-        <is>
-          <t>What method was used for sequencing?</t>
-        </is>
-      </c>
-      <c r="C344" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="D344" t="inlineStr">
-        <is>
-          <t>Sanger sequencing</t>
-        </is>
-      </c>
-      <c r="E344" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="345">
-      <c r="A345" t="inlineStr">
-        <is>
-          <t>41093949</t>
-        </is>
-      </c>
-      <c r="B345" t="inlineStr">
-        <is>
-          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
-        </is>
-      </c>
-      <c r="C345" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="D345" t="inlineStr">
-        <is>
-          <t>NRTIs, NNRTIs</t>
-        </is>
-      </c>
-      <c r="E345" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="346">
-      <c r="A346" t="inlineStr">
-        <is>
-          <t>41093949</t>
-        </is>
-      </c>
-      <c r="B346" t="inlineStr">
-        <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
-        </is>
-      </c>
-      <c r="C346" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="D346" t="inlineStr">
-        <is>
-          <t>NRTI: azvudine, zidovudine, lamivudine, tenofovir DF, abacavir, emtricitabine; NNRTI: nevirapine, etravirine, efavirenz</t>
-        </is>
-      </c>
-      <c r="E346" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="347">
-      <c r="A347" t="inlineStr">
-        <is>
-          <t>41112839</t>
-        </is>
-      </c>
-      <c r="B347" t="inlineStr">
-        <is>
-          <t>What were the GenBank accession numbers for sequenced HIV isolates?</t>
-        </is>
-      </c>
-      <c r="C347" t="inlineStr">
-        <is>
-          <t>PP280627- PP280757</t>
-        </is>
-      </c>
-      <c r="D347" t="inlineStr">
-        <is>
-          <t>PP280627 to PP280757</t>
-        </is>
-      </c>
-      <c r="E347" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="348">
-      <c r="A348" t="inlineStr">
-        <is>
-          <t>41112839</t>
-        </is>
-      </c>
-      <c r="B348" t="inlineStr">
-        <is>
-          <t>What method was used for sequencing?</t>
-        </is>
-      </c>
-      <c r="C348" t="inlineStr">
-        <is>
-          <t>Sanger</t>
-        </is>
-      </c>
-      <c r="D348" t="inlineStr">
-        <is>
-          <t>Big Dye Terminator v3.1 and ABI 3100 Avant sequencer</t>
-        </is>
-      </c>
-      <c r="E348" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="349">
-      <c r="A349" t="inlineStr">
-        <is>
-          <t>41129268</t>
-        </is>
-      </c>
-      <c r="B349" t="inlineStr">
-        <is>
-          <t>Does the paper report in vitro drug susceptibility data?</t>
-        </is>
-      </c>
-      <c r="C349" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D349" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E349" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="350">
-      <c r="A350" t="inlineStr">
-        <is>
-          <t>41130593</t>
-        </is>
-      </c>
-      <c r="B350" t="inlineStr">
-        <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
-        </is>
-      </c>
-      <c r="C350" t="n">
-        <v>64</v>
-      </c>
-      <c r="D350" t="inlineStr">
-        <is>
-          <t>53</t>
-        </is>
-      </c>
-      <c r="E350" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="351">
-      <c r="A351" t="inlineStr">
-        <is>
-          <t>41130593</t>
-        </is>
-      </c>
-      <c r="B351" t="inlineStr">
-        <is>
-          <t>From which countries were the sequenced samples obtained?</t>
-        </is>
-      </c>
-      <c r="C351" t="inlineStr">
-        <is>
-          <t>Not provided (multicenter trial)</t>
-        </is>
-      </c>
-      <c r="D351" t="inlineStr">
-        <is>
-          <t>South Africa</t>
-        </is>
-      </c>
-      <c r="E351" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="352">
-      <c r="A352" t="inlineStr">
-        <is>
-          <t>41130593</t>
-        </is>
-      </c>
-      <c r="B352" t="inlineStr">
-        <is>
-          <t>From what years were the sequenced samples obtained?</t>
-        </is>
-      </c>
-      <c r="C352" t="inlineStr">
-        <is>
-          <t>Not provided</t>
-        </is>
-      </c>
-      <c r="D352" t="inlineStr">
-        <is>
-          <t>2021 to 2023</t>
-        </is>
-      </c>
-      <c r="E352" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="353">
-      <c r="A353" t="inlineStr">
-        <is>
-          <t>41130593</t>
-        </is>
-      </c>
-      <c r="B353" t="inlineStr">
-        <is>
-          <t>Were samples cloned prior to sequencing?</t>
-        </is>
-      </c>
-      <c r="C353" t="inlineStr">
-        <is>
-          <t>Yes (single genome)</t>
-        </is>
-      </c>
-      <c r="D353" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E353" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="354">
-      <c r="A354" t="inlineStr">
-        <is>
-          <t>41130593</t>
-        </is>
-      </c>
-      <c r="B354" t="inlineStr">
-        <is>
-          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
-        </is>
-      </c>
-      <c r="C354" t="inlineStr">
-        <is>
-          <t>NRTI, CAI</t>
-        </is>
-      </c>
-      <c r="D354" t="inlineStr">
-        <is>
-          <t>NRTIs, NNRTIs.</t>
-        </is>
-      </c>
-      <c r="E354" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="355">
-      <c r="A355" t="inlineStr">
-        <is>
-          <t>41140464</t>
-        </is>
-      </c>
-      <c r="B355" t="inlineStr">
-        <is>
-          <t>From what years were the sequenced samples obtained?</t>
-        </is>
-      </c>
-      <c r="C355" t="inlineStr">
-        <is>
-          <t>Not available (deposited 2015-2025)</t>
-        </is>
-      </c>
-      <c r="D355" t="inlineStr">
-        <is>
-          <t>2015-2025</t>
-        </is>
-      </c>
-      <c r="E355" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="356">
-      <c r="A356" t="inlineStr">
-        <is>
-          <t>41140464</t>
-        </is>
-      </c>
-      <c r="B356" t="inlineStr">
-        <is>
-          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
-        </is>
-      </c>
-      <c r="C356" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D356" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E356" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="357">
-      <c r="A357" t="inlineStr">
-        <is>
-          <t>41140464</t>
-        </is>
-      </c>
-      <c r="B357" t="inlineStr">
-        <is>
-          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
-        </is>
-      </c>
-      <c r="C357" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D357" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E357" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="358">
-      <c r="A358" t="inlineStr">
-        <is>
-          <t>41140464</t>
-        </is>
-      </c>
-      <c r="B358" t="inlineStr">
-        <is>
-          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
-        </is>
-      </c>
-      <c r="C358" t="inlineStr">
-        <is>
-          <t>NRTI, NNRTI, PI, INSTI</t>
-        </is>
-      </c>
-      <c r="D358" t="inlineStr">
-        <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="E358" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update evals with 8B corrections
</commit_message>
<xml_diff>
--- a/eval/learning-curve/results/learning_curve_gpt-4o_ft200_incorrect.xlsx
+++ b/eval/learning-curve/results/learning_curve_gpt-4o_ft200_incorrect.xlsx
@@ -488,17 +488,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Were samples cloned prior to sequencing?</t>
+          <t>What method was used for sequencing?</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sanger</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="E3" t="n">
@@ -513,15 +513,19 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
+          <t>Were samples cloned prior to sequencing?</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>IN</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
@@ -534,19 +538,15 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>What method was used for sequencing?</t>
+          <t>Which HIV genes were reported to have been sequenced?</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Sanger</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Not specified</t>
-        </is>
-      </c>
+          <t>IN</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="n">
         <v>0</v>
       </c>
@@ -634,17 +634,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>From which countries were the sequenced samples obtained?</t>
+          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -659,17 +659,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
+          <t>From which countries were the sequenced samples obtained?</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="E10" t="n">
@@ -684,7 +684,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
+          <t>What type of samples were sequenced?</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -694,7 +694,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>RT</t>
+          <t>Virus isolates</t>
         </is>
       </c>
       <c r="E11" t="n">
@@ -709,7 +709,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>What type of samples were sequenced?</t>
+          <t>Which HIV genes were reported to have been sequenced?</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -719,7 +719,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Virus isolates</t>
+          <t>RT</t>
         </is>
       </c>
       <c r="E12" t="n">
@@ -809,17 +809,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Were sequences from the paper made publicly available?</t>
+          <t>What type of samples were sequenced?</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>PBMC, Plasma</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>plasma RNA</t>
         </is>
       </c>
       <c r="E16" t="n">
@@ -834,17 +834,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>What type of samples were sequenced?</t>
+          <t>Were sequences from the paper made publicly available?</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>PBMC, Plasma</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>plasma RNA</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E17" t="n">
@@ -884,17 +884,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>NRTIs, NNRTIs</t>
         </is>
       </c>
       <c r="E19" t="n">
@@ -909,17 +909,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>RT</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>gag-pol</t>
+          <t>Abacavir (ABC), Didanosine (ddI), Emtricitabine (FTC), Lamivudine (3TC), Zidovudine (ZDV), Stavudine (d4T),Tenofovir disoproxil fumarate (TDF), Nevirapine (NVP), Efavirenz (EFV), Etravirine (ETR), Rilpivirine (RPV)</t>
         </is>
       </c>
       <c r="E20" t="n">
@@ -934,17 +934,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>51</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>NRTIs, NNRTIs</t>
+          <t>42</t>
         </is>
       </c>
       <c r="E21" t="n">
@@ -959,17 +959,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+          <t>Which HIV genes were reported to have been sequenced?</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>RT</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Abacavir (ABC), Didanosine (ddI), Emtricitabine (FTC), Lamivudine (3TC), Zidovudine (ZDV), Stavudine (d4T),Tenofovir disoproxil fumarate (TDF), Nevirapine (NVP), Efavirenz (EFV), Etravirine (ETR), Rilpivirine (RPV)</t>
+          <t>gag-pol</t>
         </is>
       </c>
       <c r="E22" t="n">
@@ -1059,17 +1059,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Were sequences from the paper made publicly available?</t>
+          <t>What method was used for sequencing?</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sanger sequencing</t>
         </is>
       </c>
       <c r="E26" t="n">
@@ -1084,17 +1084,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Were samples cloned prior to sequencing?</t>
+          <t>What type of samples were sequenced?</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>viral isolates</t>
         </is>
       </c>
       <c r="E27" t="n">
@@ -1109,17 +1109,17 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>What method was used for sequencing?</t>
+          <t>Were sequences from the paper made publicly available?</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Sanger sequencing</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E28" t="n">
@@ -1134,17 +1134,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>What type of samples were sequenced?</t>
+          <t>Were samples cloned prior to sequencing?</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>viral isolates</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E29" t="n">
@@ -1226,15 +1226,19 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
+          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>51</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="E33" t="n">
         <v>0</v>
       </c>
@@ -1247,15 +1251,19 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>From which countries were the sequenced samples obtained?</t>
+          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="E34" t="n">
         <v>0</v>
       </c>
@@ -1268,12 +1276,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>From what years were the sequenced samples obtained?</t>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2021-2022</t>
+          <t>51</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1289,12 +1297,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
+          <t>From which countries were the sequenced samples obtained?</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>RT, IN</t>
+          <t>US</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1310,19 +1318,15 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
+          <t>From what years were the sequenced samples obtained?</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+          <t>2021-2022</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
       <c r="E37" t="n">
         <v>0</v>
       </c>
@@ -1335,19 +1339,15 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
+          <t>Which HIV genes were reported to have been sequenced?</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+          <t>RT, IN</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
       <c r="E38" t="n">
         <v>0</v>
       </c>
@@ -1385,17 +1385,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
+          <t>What type of samples were sequenced?</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>Plasma</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="E40" t="n">
@@ -1410,17 +1410,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>From which countries were the sequenced samples obtained?</t>
+          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>UK, USA, Belgium, Canada, Netherlands, Switzerland, Portugal, Italy, South Korea, Spain</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Not applicable</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -1435,17 +1435,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>From what years were the sequenced samples obtained?</t>
+          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2016-2020</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Not applicable</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="E42" t="n">
@@ -1460,17 +1460,17 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>RT, IN</t>
+          <t>CAB, RPV</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>cobicistat-boosted darunavir, tenofovir alafenamide, emtricitabine, dolutegravir</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -1485,17 +1485,17 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>What type of samples were sequenced?</t>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Plasma</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E44" t="n">
@@ -1510,17 +1510,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
+          <t>From which countries were the sequenced samples obtained?</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>UK, USA, Belgium, Canada, Netherlands, Switzerland, Portugal, Italy, South Korea, Spain</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>Not applicable</t>
         </is>
       </c>
       <c r="E45" t="n">
@@ -1535,17 +1535,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
+          <t>From what years were the sequenced samples obtained?</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>2016-2020</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>Not applicable</t>
         </is>
       </c>
       <c r="E46" t="n">
@@ -1560,17 +1560,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+          <t>Which HIV genes were reported to have been sequenced?</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>CAB, RPV</t>
+          <t>RT, IN</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>cobicistat-boosted darunavir, tenofovir alafenamide, emtricitabine, dolutegravir</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="E47" t="n">
@@ -1685,17 +1685,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>TDF,FTC,EVG</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>EFV, RPV, ETR, ATV/r, SQV/r, DRV/r, RAL, DTG, AZT, TDF, 3TC, FTC</t>
         </is>
       </c>
       <c r="E52" t="n">
@@ -1710,17 +1710,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>TDF,FTC,EVG</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>EFV, RPV, ETR, ATV/r, SQV/r, DRV/r, RAL, DTG, AZT, TDF, 3TC, FTC</t>
+          <t>13</t>
         </is>
       </c>
       <c r="E53" t="n">
@@ -1760,17 +1760,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
+          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>120 * 76% = 95, or 120 or 129</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="E55" t="n">
@@ -1785,17 +1785,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>From which countries were the sequenced samples obtained?</t>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>120 * 76% = 95, or 120 or 129</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Not applicable</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E56" t="n">
@@ -1810,17 +1810,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
+          <t>From which countries were the sequenced samples obtained?</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>RT, IN</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Not applicable</t>
         </is>
       </c>
       <c r="E57" t="n">
@@ -1835,17 +1835,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
+          <t>Which HIV genes were reported to have been sequenced?</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>RT, IN</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="E58" t="n">
@@ -1885,15 +1885,19 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
+          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>14</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="E60" t="n">
         <v>0</v>
       </c>
@@ -1906,15 +1910,19 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>From which countries were the sequenced samples obtained?</t>
+          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>France</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr"/>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="E61" t="n">
         <v>0</v>
       </c>
@@ -1927,12 +1935,12 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>From what years were the sequenced samples obtained?</t>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2019-2020</t>
+          <t>NRTI, INSTI</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -1948,12 +1956,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>RT, IN</t>
+          <t>BIC, FTC, TAF</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
@@ -1969,19 +1977,15 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
       <c r="E64" t="n">
         <v>0</v>
       </c>
@@ -1994,19 +1998,15 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
+          <t>From which countries were the sequenced samples obtained?</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
+          <t>France</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
       <c r="E65" t="n">
         <v>0</v>
       </c>
@@ -2019,12 +2019,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+          <t>From what years were the sequenced samples obtained?</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>NRTI, INSTI</t>
+          <t>2019-2020</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -2040,12 +2040,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+          <t>Which HIV genes were reported to have been sequenced?</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>BIC, FTC, TAF</t>
+          <t>RT, IN</t>
         </is>
       </c>
       <c r="D67" t="inlineStr"/>
@@ -2086,12 +2086,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>8 and 10</t>
+          <t>NNRTI, INSTI</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2111,12 +2111,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>RT, IN</t>
+          <t>CAB, RPV</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2136,12 +2136,12 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>NNRTI, INSTI</t>
+          <t>8 and 10</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2161,12 +2161,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+          <t>Which HIV genes were reported to have been sequenced?</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>CAB, RPV</t>
+          <t>RT, IN</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2236,17 +2236,17 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
+          <t>What type of samples were sequenced?</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>62 or 3</t>
+          <t>Plasma</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>The paper does not specify how many individuals had samples obtained for HIV sequencing.</t>
+          <t>The paper does not specify the type of samples that were sequenced.</t>
         </is>
       </c>
       <c r="E75" t="n">
@@ -2261,17 +2261,17 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>RT, IN</t>
+          <t>TDF, 3TC, FTC, EFV, NVP, DTG</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>The paper does not specify which HIV genes were sequenced.</t>
+          <t>The individuals received tenofovir, lamivudine/emtricitabine, and an NNRTI (efavirenz or nevirapine) before sample sequencing.</t>
         </is>
       </c>
       <c r="E76" t="n">
@@ -2286,17 +2286,17 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>What type of samples were sequenced?</t>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Plasma</t>
+          <t>62 or 3</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>The paper does not specify the type of samples that were sequenced.</t>
+          <t>The paper does not specify how many individuals had samples obtained for HIV sequencing.</t>
         </is>
       </c>
       <c r="E77" t="n">
@@ -2311,17 +2311,17 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+          <t>Which HIV genes were reported to have been sequenced?</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>TDF, 3TC, FTC, EFV, NVP, DTG</t>
+          <t>RT, IN</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>The individuals received tenofovir, lamivudine/emtricitabine, and an NNRTI (efavirenz or nevirapine) before sample sequencing.</t>
+          <t>The paper does not specify which HIV genes were sequenced.</t>
         </is>
       </c>
       <c r="E78" t="n">
@@ -2336,17 +2336,17 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
+          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>527</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>594</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E79" t="n">
@@ -2361,7 +2361,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>From what years were the sequenced samples obtained?</t>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2371,7 +2371,7 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Data as of August 2021</t>
+          <t>NRTI, NNRTI, PI</t>
         </is>
       </c>
       <c r="E80" t="n">
@@ -2386,17 +2386,17 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>527</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>594</t>
         </is>
       </c>
       <c r="E81" t="n">
@@ -2411,7 +2411,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+          <t>From what years were the sequenced samples obtained?</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2421,7 +2421,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>NRTI, NNRTI, PI</t>
+          <t>Data as of August 2021</t>
         </is>
       </c>
       <c r="E82" t="n">
@@ -2586,12 +2586,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
+          <t>What type of samples were sequenced?</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>RT</t>
+          <t>Plasma, CSF, PBMC</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -2611,12 +2611,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>What type of samples were sequenced?</t>
+          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Plasma, CSF, PBMC</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2636,17 +2636,17 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>DTG</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="E91" t="n">
@@ -2661,17 +2661,17 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+          <t>Which HIV genes were reported to have been sequenced?</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>DTG</t>
+          <t>RT</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="E92" t="n">
@@ -2832,17 +2832,17 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>From which countries were the sequenced samples obtained?</t>
+          <t>What type of samples were sequenced?</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Whole Blood, Semen</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Plasma RNA and HIV DNA</t>
         </is>
       </c>
       <c r="E99" t="n">
@@ -2857,17 +2857,17 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>What type of samples were sequenced?</t>
+          <t>From which countries were the sequenced samples obtained?</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Whole Blood, Semen</t>
+          <t>France</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Plasma RNA and HIV DNA</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="E100" t="n">
@@ -2907,17 +2907,17 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Does the paper report in vitro drug susceptibility data?</t>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>NRTIs, NNRTIs</t>
         </is>
       </c>
       <c r="E102" t="n">
@@ -2932,7 +2932,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -2942,7 +2942,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>NRTIs, NNRTIs</t>
+          <t>Dolutegravir (DTG), Emtricitabine (FTC), Tenofovir disoproxil fumarate (TDF)</t>
         </is>
       </c>
       <c r="E103" t="n">
@@ -2957,17 +2957,17 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+          <t>Does the paper report in vitro drug susceptibility data?</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Dolutegravir (DTG), Emtricitabine (FTC), Tenofovir disoproxil fumarate (TDF)</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E104" t="n">
@@ -3182,17 +3182,17 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
+          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>1651</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E113" t="n">
@@ -3207,17 +3207,17 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
+          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>RT</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E114" t="n">
@@ -3232,17 +3232,17 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NNRTI, INSTI</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="E115" t="n">
@@ -3257,17 +3257,17 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>CAB, RPV</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="E116" t="n">
@@ -3282,12 +3282,12 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>NNRTI, INSTI</t>
+          <t>1651</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -3307,12 +3307,12 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+          <t>Which HIV genes were reported to have been sequenced?</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>CAB, RPV</t>
+          <t>RT</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -3507,17 +3507,17 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>What were the GenBank accession numbers for sequenced HIV isolates?</t>
+          <t>What method was used for sequencing?</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>Sanger sequencing, Illumina sequencing</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>K03455</t>
+          <t>Next-Generation Sequencing (NGS)</t>
         </is>
       </c>
       <c r="E126" t="n">
@@ -3532,17 +3532,17 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>NFLG</t>
+          <t>DTG</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Gag, Pol, Env, Integnase RT</t>
+          <t>1. NRTIs: FTC, TDF, ABC, ZDV, 3TC, D4T 2. NNRTIs: RPV, NVP, EFV 3. PIs: LPV/RTV, DRV/RTV, IDV 4. INSTIs: RAL, ETV</t>
         </is>
       </c>
       <c r="E127" t="n">
@@ -3557,17 +3557,17 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>What method was used for sequencing?</t>
+          <t>What were the GenBank accession numbers for sequenced HIV isolates?</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Sanger sequencing, Illumina sequencing</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Next-Generation Sequencing (NGS)</t>
+          <t>K03455</t>
         </is>
       </c>
       <c r="E128" t="n">
@@ -3582,17 +3582,17 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+          <t>Which HIV genes were reported to have been sequenced?</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>DTG</t>
+          <t>NFLG</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>1. NRTIs: FTC, TDF, ABC, ZDV, 3TC, D4T 2. NNRTIs: RPV, NVP, EFV 3. PIs: LPV/RTV, DRV/RTV, IDV 4. INSTIs: RAL, ETV</t>
+          <t>Gag, Pol, Env, Integnase RT</t>
         </is>
       </c>
       <c r="E129" t="n">
@@ -3632,17 +3632,17 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
+          <t>What method was used for sequencing?</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>379</t>
+          <t>Sanger sequencing</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>391</t>
+          <t>ABI 3500</t>
         </is>
       </c>
       <c r="E131" t="n">
@@ -3657,17 +3657,17 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>What method was used for sequencing?</t>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Sanger sequencing</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>ABI 3500</t>
+          <t>NRTIs, NNRTIs</t>
         </is>
       </c>
       <c r="E132" t="n">
@@ -3682,17 +3682,17 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>379</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>NRTIs, NNRTIs</t>
+          <t>391</t>
         </is>
       </c>
       <c r="E133" t="n">
@@ -3707,7 +3707,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Were sequences from the paper made publicly available?</t>
+          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -3732,17 +3732,17 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>INSTI</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>NRTI, NNRTI, PI</t>
         </is>
       </c>
       <c r="E135" t="n">
@@ -3757,17 +3757,17 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>INSTI</t>
+          <t>DTG</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>NRTI, NNRTI, PI</t>
+          <t>EFV, ATV, FTC, TDF</t>
         </is>
       </c>
       <c r="E136" t="n">
@@ -3782,17 +3782,17 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+          <t>Were sequences from the paper made publicly available?</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>DTG</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>EFV, ATV, FTC, TDF</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E137" t="n">
@@ -3807,17 +3807,17 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Were sequences from the paper made publicly available?</t>
+          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
           <t>No</t>
-        </is>
-      </c>
-      <c r="D138" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
       <c r="E138" t="n">
@@ -3832,7 +3832,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
+          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -3857,17 +3857,17 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
+          <t>Were sequences from the paper made publicly available?</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="D140" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
       <c r="E140" t="n">
@@ -3982,17 +3982,17 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>From which countries were the sequenced samples obtained?</t>
+          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Botswana, South Africa, Thailand, and the U.S.</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E145" t="n">
@@ -4007,17 +4007,17 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>From what years were the sequenced samples obtained?</t>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2020-2021</t>
+          <t>PI, INSTI</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>NRTI, INSTI</t>
         </is>
       </c>
       <c r="E146" t="n">
@@ -4032,17 +4032,17 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>RT</t>
+          <t>LPV, DTG, RAL, ABC, 3TC</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>Lopinavir/ritonavir, dolutegravir, raltegravir</t>
         </is>
       </c>
       <c r="E147" t="n">
@@ -4057,17 +4057,17 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
+          <t>From which countries were the sequenced samples obtained?</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Botswana, South Africa, Thailand, and the U.S.</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="E148" t="n">
@@ -4082,17 +4082,17 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+          <t>From what years were the sequenced samples obtained?</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>PI, INSTI</t>
+          <t>2020-2021</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>NRTI, INSTI</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="E149" t="n">
@@ -4107,17 +4107,17 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+          <t>Which HIV genes were reported to have been sequenced?</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>LPV, DTG, RAL, ABC, 3TC</t>
+          <t>RT</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Lopinavir/ritonavir, dolutegravir, raltegravir</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="E150" t="n">
@@ -4157,17 +4157,17 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
+          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E152" t="n">
@@ -4182,15 +4182,19 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
+          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>RT</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr"/>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
       <c r="E153" t="n">
         <v>0</v>
       </c>
@@ -4203,17 +4207,17 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NRTI, NNRTI, PI</t>
         </is>
       </c>
       <c r="E154" t="n">
@@ -4228,17 +4232,17 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Tenofovir, Lamivudine, Emtricitabine, Abacavir, Efavirenz, Etravirine, Dolutegravir, Darunavir, Ritonavir</t>
         </is>
       </c>
       <c r="E155" t="n">
@@ -4253,17 +4257,17 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>1</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>NRTI, NNRTI, PI</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E156" t="n">
@@ -4278,19 +4282,15 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+          <t>Which HIV genes were reported to have been sequenced?</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Not reported</t>
-        </is>
-      </c>
-      <c r="D157" t="inlineStr">
-        <is>
-          <t>Tenofovir, Lamivudine, Emtricitabine, Abacavir, Efavirenz, Etravirine, Dolutegravir, Darunavir, Ritonavir</t>
-        </is>
-      </c>
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr"/>
       <c r="E157" t="n">
         <v>0</v>
       </c>
@@ -4303,17 +4303,17 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Were sequences from the paper made publicly available?</t>
+          <t>What type of samples were sequenced?</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Plasma</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not specified</t>
         </is>
       </c>
       <c r="E158" t="n">
@@ -4328,17 +4328,17 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>What type of samples were sequenced?</t>
+          <t>Were sequences from the paper made publicly available?</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Plasma</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Not specified</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E159" t="n">
@@ -4353,17 +4353,17 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
+          <t>What method was used for sequencing?</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>551</t>
+          <t>Sanger sequencing</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>554</t>
+          <t>ABI-3730 DNA genetic analyzer</t>
         </is>
       </c>
       <c r="E160" t="n">
@@ -4378,17 +4378,17 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>What method was used for sequencing?</t>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Sanger sequencing</t>
+          <t>551</t>
         </is>
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>ABI-3730 DNA genetic analyzer</t>
+          <t>554</t>
         </is>
       </c>
       <c r="E161" t="n">
@@ -4478,17 +4478,17 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Were sequences from the paper made publicly available?</t>
+          <t>What method was used for sequencing?</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Sanger sequencing</t>
         </is>
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>ABI 3730XL</t>
         </is>
       </c>
       <c r="E165" t="n">
@@ -4503,17 +4503,17 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>What method was used for sequencing?</t>
+          <t>Were sequences from the paper made publicly available?</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Sanger sequencing</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>ABI 3730XL</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E166" t="n">
@@ -4553,17 +4553,17 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>From which countries were the sequenced samples obtained?</t>
+          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Not applicable</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E168" t="n">
@@ -4578,12 +4578,12 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>From what years were the sequenced samples obtained?</t>
+          <t>From which countries were the sequenced samples obtained?</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>2020-2021</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="D169" t="inlineStr">
@@ -4603,12 +4603,12 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
+          <t>From what years were the sequenced samples obtained?</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>RT, IN</t>
+          <t>2020-2021</t>
         </is>
       </c>
       <c r="D170" t="inlineStr">
@@ -4628,17 +4628,17 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
+          <t>Which HIV genes were reported to have been sequenced?</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>RT, IN</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Not applicable</t>
         </is>
       </c>
       <c r="E171" t="n">
@@ -4753,15 +4753,19 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
+          <t>What type of samples were sequenced?</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>4559 and 3097</t>
-        </is>
-      </c>
-      <c r="D176" t="inlineStr"/>
+          <t>Serum, Plasma, DBS</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Plasma, serum, dried serum, or plasma spots</t>
+        </is>
+      </c>
       <c r="E176" t="n">
         <v>0</v>
       </c>
@@ -4774,19 +4778,15 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>What type of samples were sequenced?</t>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Serum, Plasma, DBS</t>
-        </is>
-      </c>
-      <c r="D177" t="inlineStr">
-        <is>
-          <t>Plasma, serum, dried serum, or plasma spots</t>
-        </is>
-      </c>
+          <t>4559 and 3097</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr"/>
       <c r="E177" t="n">
         <v>0</v>
       </c>
@@ -4799,17 +4799,17 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
+          <t>What type of samples were sequenced?</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>NFLG, Envelope</t>
+          <t>PBMC</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>env</t>
+          <t>plasma viral RNA</t>
         </is>
       </c>
       <c r="E178" t="n">
@@ -4824,17 +4824,17 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>What type of samples were sequenced?</t>
+          <t>Which HIV genes were reported to have been sequenced?</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>PBMC</t>
+          <t>NFLG, Envelope</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>plasma viral RNA</t>
+          <t>env</t>
         </is>
       </c>
       <c r="E179" t="n">
@@ -4874,17 +4874,17 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Were sequences from the paper made publicly available?</t>
+          <t>What method was used for sequencing?</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sanger sequencing</t>
         </is>
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>PCR products were sequenced using the Applied Biosystems 3500 genetic analyzer</t>
         </is>
       </c>
       <c r="E181" t="n">
@@ -4899,17 +4899,17 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>What method was used for sequencing?</t>
+          <t>Were sequences from the paper made publicly available?</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Sanger sequencing</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>PCR products were sequenced using the Applied Biosystems 3500 genetic analyzer</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E182" t="n">
@@ -5124,17 +5124,17 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
+          <t>What type of samples were sequenced?</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>820 or 46</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>Plasma</t>
         </is>
       </c>
       <c r="E191" t="n">
@@ -5149,17 +5149,17 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>What type of samples were sequenced?</t>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>820 or 46</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Plasma</t>
+          <t>48</t>
         </is>
       </c>
       <c r="E192" t="n">
@@ -5349,17 +5349,17 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Does the paper report in vitro drug susceptibility data?</t>
+          <t>What type of samples were sequenced?</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>The paper mentions that amino acid sequences of HIV enzymes were used.</t>
         </is>
       </c>
       <c r="E200" t="n">
@@ -5374,17 +5374,17 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Were sequences from the paper made publicly available?</t>
+          <t>Does the paper report in vitro drug susceptibility data?</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
           <t>Yes</t>
-        </is>
-      </c>
-      <c r="D201" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
       <c r="E201" t="n">
@@ -5399,17 +5399,17 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
+          <t>Were sequences from the paper made publicly available?</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>The paper mentions the sequencing of protease and reverse transcriptase genes.</t>
+          <t>No</t>
         </is>
       </c>
       <c r="E202" t="n">
@@ -5424,7 +5424,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>What type of samples were sequenced?</t>
+          <t>Which HIV genes were reported to have been sequenced?</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -5434,7 +5434,7 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>The paper mentions that amino acid sequences of HIV enzymes were used.</t>
+          <t>The paper mentions the sequencing of protease and reverse transcriptase genes.</t>
         </is>
       </c>
       <c r="E203" t="n">
@@ -5574,17 +5574,17 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
+          <t>What type of samples were sequenced?</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>PR, RT, IN</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>HIV from plasma</t>
         </is>
       </c>
       <c r="E209" t="n">
@@ -5599,17 +5599,17 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>What type of samples were sequenced?</t>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>NRTI, NNRTI, PI, INSTI</t>
         </is>
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>HIV from plasma</t>
+          <t>NRTIs, NNRTIs, Protease Inhibitors</t>
         </is>
       </c>
       <c r="E210" t="n">
@@ -5624,17 +5624,17 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+          <t>Which HIV genes were reported to have been sequenced?</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>NRTI, NNRTI, PI, INSTI</t>
+          <t>PR, RT, IN</t>
         </is>
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>NRTIs, NNRTIs, Protease Inhibitors</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="E211" t="n">
@@ -5674,12 +5674,12 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
+          <t>What type of samples were sequenced?</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>Plasma, PBMC</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
@@ -5699,12 +5699,12 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>From which countries were the sequenced samples obtained?</t>
+          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Italy</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D214" t="inlineStr">
@@ -5724,12 +5724,12 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>From what years were the sequenced samples obtained?</t>
+          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>2019-2020</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="D215" t="inlineStr">
@@ -5749,12 +5749,12 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>RT, IN</t>
+          <t>NRTI, NNRTI, PI, INSTI</t>
         </is>
       </c>
       <c r="D216" t="inlineStr">
@@ -5774,12 +5774,12 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>What type of samples were sequenced?</t>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Plasma, PBMC</t>
+          <t>BIC, FTC, TAF, EVG</t>
         </is>
       </c>
       <c r="D217" t="inlineStr">
@@ -5799,12 +5799,12 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Were any sequences obtained from individuals with virological failure on a treatment regimen?</t>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D218" t="inlineStr">
@@ -5824,12 +5824,12 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
+          <t>From which countries were the sequenced samples obtained?</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Italy</t>
         </is>
       </c>
       <c r="D219" t="inlineStr">
@@ -5849,12 +5849,12 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+          <t>From what years were the sequenced samples obtained?</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>NRTI, NNRTI, PI, INSTI</t>
+          <t>2019-2020</t>
         </is>
       </c>
       <c r="D220" t="inlineStr">
@@ -5874,12 +5874,12 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+          <t>Which HIV genes were reported to have been sequenced?</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>BIC, FTC, TAF, EVG</t>
+          <t>RT, IN</t>
         </is>
       </c>
       <c r="D221" t="inlineStr">
@@ -5899,17 +5899,17 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>What were the GenBank accession numbers for sequenced HIV isolates?</t>
+          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>K03455</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E222" t="n">
@@ -5924,17 +5924,17 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NRTIs, NNRTIs, PIs</t>
         </is>
       </c>
       <c r="E223" t="n">
@@ -5949,7 +5949,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+          <t>What were the GenBank accession numbers for sequenced HIV isolates?</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -5959,7 +5959,7 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>NRTIs, NNRTIs, PIs</t>
+          <t>K03455</t>
         </is>
       </c>
       <c r="E224" t="n">
@@ -5974,17 +5974,17 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>From which countries were the sequenced samples obtained?</t>
+          <t>What type of samples were sequenced?</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>Plasma</t>
         </is>
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="E225" t="n">
@@ -5999,17 +5999,17 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>What type of samples were sequenced?</t>
+          <t>From which countries were the sequenced samples obtained?</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>Plasma</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="E226" t="n">
@@ -6024,17 +6024,17 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>How many individuals had samples obtained for HIV sequencing?</t>
+          <t>What method was used for sequencing?</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>NGS</t>
         </is>
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>195</t>
+          <t>High-throughput sequencing</t>
         </is>
       </c>
       <c r="E227" t="n">
@@ -6049,17 +6049,17 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>What method was used for sequencing?</t>
+          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>NGS</t>
+          <t>No</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>High-throughput sequencing</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="E228" t="n">
@@ -6074,17 +6074,17 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>Does the paper report HIV sequences from individuals who had previously received ARV drugs?</t>
+          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>NRTI, PI, NNRTI</t>
         </is>
       </c>
       <c r="E229" t="n">
@@ -6099,7 +6099,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>Which drug classes were received by individuals in the study before sample sequencing?</t>
+          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -6109,7 +6109,7 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>NRTI, PI, NNRTI</t>
+          <t>EFV, NVP, AZT, 3TC, tenofovir, abacavir</t>
         </is>
       </c>
       <c r="E230" t="n">
@@ -6124,17 +6124,17 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>Which drugs were received by individuals in the study before sample sequencing?</t>
+          <t>How many individuals had samples obtained for HIV sequencing?</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>37</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>EFV, NVP, AZT, 3TC, tenofovir, abacavir</t>
+          <t>195</t>
         </is>
       </c>
       <c r="E231" t="n">
@@ -6174,17 +6174,17 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Which HIV genes were reported to have been sequenced?</t>
+          <t>What type of samples were sequenced?</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>RT, CA</t>
+          <t>Not reported</t>
         </is>
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>Gag, Pol</t>
+          <t>Plasma viral RNA</t>
         </is>
       </c>
       <c r="E233" t="n">
@@ -6199,17 +6199,17 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>What type of samples were sequenced?</t>
+          <t>Which HIV genes were reported to have been sequenced?</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Not reported</t>
+          <t>RT, CA</t>
         </is>
       </c>
       <c r="D234" t="inlineStr">
         <is>
-          <t>Plasma viral RNA</t>
+          <t>Gag, Pol</t>
         </is>
       </c>
       <c r="E234" t="n">

</xml_diff>